<commit_message>
Fixed SQL insertion script
</commit_message>
<xml_diff>
--- a/data/interventions.xlsx
+++ b/data/interventions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hessoit-my.sharepoint.com/personal/quentin_thuler_hes-so_ch/Documents/Bureau/HEIG Cloud/InfraDon/Projet/comem-infradon/projet/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hessoit-my.sharepoint.com/personal/quentin_thuler_hes-so_ch/Documents/Bureau/HEIG Cloud/InfraDon/Projet/Travail Groupe/InfraDon-Group-Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_3D455F0417EA723B4183DCF0505ED87656CC8B29" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2687CF5-8384-4A91-8A75-BC9D93FE661C}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_3D455F0417EA723B4183DCF0505ED87656CC8B29" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90F917AC-45F1-46A8-AC5D-75B634AE6052}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1457,6 +1457,9 @@
   <dimension ref="A1:G151"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
+    <col min="1" max="1" width="9.9296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.1328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.73046875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.73046875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21.86328125" bestFit="1" customWidth="1"/>

</xml_diff>